<commit_message>
scan: seg7 2026-10-26 15:54 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq8_2026-10-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>69.94965166998817</v>
+        <v>69.94965175462735</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>19.19329778752608</v>
+        <v>19.19329802336328</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>7.940162131896488</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.3163592926895054</v>
+        <v>0.3163592924948281</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>68.03869776481109</v>
+        <v>68.03869779931199</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>21.28026601628239</v>
+        <v>21.28026604239151</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.504310862823595</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1.052771919587448</v>
+        <v>1.052771918549143</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>74.45730781170458</v>
+        <v>74.45730782053397</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>39.0104089967719</v>
+        <v>39.0104089987615</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.722705245415632</v>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>59.33528991038312</v>
+        <v>59.33528986086874</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>24.76698911978846</v>
+        <v>24.76698919142567</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>7.622238109654431</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.163103766224757</v>
+        <v>1.163103766354558</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>70.83526071726669</v>
+        <v>70.83526072578613</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>52.33623119440794</v>
+        <v>52.3362311663102</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>4.641489785575262</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>3.030560989705133</v>
+        <v>3.030560989834909</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -803,7 +803,7 @@
         <v/>
       </c>
       <c r="D7" s="2" t="n">
-        <v>788.0657424137028</v>
+        <v>788.0657424137029</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>346</v>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>62.18592551304516</v>
+        <v>62.1859254895444</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>29.19834304703508</v>
+        <v>29.19834311325341</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.217630350492084</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.710352955460622</v>
+        <v>1.710352958835055</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>783.1688664672788</v>
+        <v>783.1688664672783</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>420</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>64.30031513783889</v>
+        <v>64.3003150505638</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>37.03299659184595</v>
+        <v>37.03299660972345</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.604068862259369</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>5.203575769660699</v>
+        <v>5.203575770439357</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>67.34293753263336</v>
+        <v>67.34293755549697</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>62.76794308974016</v>
+        <v>62.76794308880867</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.6413756187117383</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-2.676979815211666</v>
+        <v>-2.67697981547127</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>54.72480170258331</v>
+        <v>54.7248016368945</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>26.90033099992017</v>
+        <v>26.9003311091649</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.150892226377595</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-5.853934577641549</v>
+        <v>-5.85393457660328</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>53.19198548856367</v>
+        <v>53.19198551361392</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>24.06601552175643</v>
+        <v>24.06601552382029</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.34306299199178</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.6402986362402208</v>
+        <v>-0.6402986371487178</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>56.31363704471918</v>
+        <v>56.31363707311227</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>32.75928367151509</v>
+        <v>32.75928343774675</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.042011461143822</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.669609865712558</v>
+        <v>-0.6696098661538343</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>631.3528161692608</v>
+        <v>631.352816169261</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>24.95</v>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>57.47428918148973</v>
+        <v>57.47428873134015</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>17.20984157133817</v>
+        <v>17.20984192539955</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.691032403918613</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.1692508148162314</v>
+        <v>0.1692508146734619</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>601.8227936948316</v>
+        <v>601.8227936948315</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>294.5</v>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>52.5376961275653</v>
+        <v>52.53769618541418</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>18.42807164009161</v>
+        <v>18.42807184930868</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.9261545656685027</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.4446222581510346</v>
+        <v>0.4446222571126914</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>63.57272341069515</v>
+        <v>63.5727237145042</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>27.71466386217884</v>
+        <v>27.71466386217883</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.895021888780528</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.9639298299164247</v>
+        <v>0.9639298282551487</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>56.92213957716753</v>
+        <v>56.92213959713399</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>29.32510521052929</v>
+        <v>29.3251052955181</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>1.188244001203</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.8388928743632311</v>
+        <v>0.838892873662398</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>52.74685582508335</v>
+        <v>52.74685587979288</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>46.44135779492929</v>
+        <v>46.44135771463289</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.6281562191566618</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-5.226515706670316</v>
+        <v>-5.226515709525671</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>587.3927484592125</v>
+        <v>587.3927484592128</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>5275</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>40.83948143259135</v>
+        <v>40.83948143861321</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>14.26846168175642</v>
+        <v>14.26846172783942</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.010550192051703</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-55.80704447574817</v>
+        <v>-55.80704447964263</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>50.5719728348904</v>
+        <v>50.57197283127809</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>40.24573190733017</v>
+        <v>40.24573200609252</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.3216410277318243</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-0.3599697691584207</v>
+        <v>-0.3599697687560817</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>51.09637830140809</v>
+        <v>51.09637824097655</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>16.90952770341487</v>
+        <v>16.90952776231768</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>1.030996144758115</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.4254610186253648</v>
+        <v>0.4254610190147214</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>476.3138932595579</v>
+        <v>476.3138932595559</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>45.9</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>49.20573157708409</v>
+        <v>49.20573112498275</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>12.52309828906167</v>
+        <v>12.52309821182338</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.5902387289890044</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.2250852716290416</v>
+        <v>0.2250852720962755</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>471.7131468764721</v>
+        <v>471.7131468764723</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>158</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>37.91715385742545</v>
+        <v>37.91715399898477</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>13.56403178611731</v>
+        <v>13.56403198373947</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.6650754418188766</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-0.6837150969125085</v>
+        <v>-0.6837150996380408</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>43.19175133161879</v>
+        <v>43.19175202554241</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>27.17915767357765</v>
+        <v>27.17915790035438</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>1.711396644695686</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.1576494219907803</v>
+        <v>-0.1576494230550256</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>459.6270241187326</v>
+        <v>459.6270241187337</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>48.5</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>58.01707422218733</v>
+        <v>58.01707416274689</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>39.61825297268022</v>
+        <v>39.61825314176064</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>3.122163418376172</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.5196112410235154</v>
+        <v>0.5196112413479834</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>449.4834192354286</v>
+        <v>449.4834192354285</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>39.2</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>52.19316828631731</v>
+        <v>52.19316830289503</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>6.517310183308232</v>
+        <v>6.517310348231315</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.5330006106749495</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.08312193244465604</v>
+        <v>0.08312193232785448</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1933,7 +1933,7 @@
         <v>44.26001799550453</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>25.43737024010688</v>
+        <v>25.43737028424433</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.2126352000985455</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-6.459398176410826</v>
+        <v>-6.459398176540606</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>35.53863545566225</v>
+        <v>35.53863552284471</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>21.62935458982821</v>
+        <v>21.62935468199205</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.6702648318182373</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-3.205462238265079</v>
+        <v>-3.20546224073101</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>45.37340788809531</v>
+        <v>45.37340792240466</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>19.59991805992352</v>
+        <v>19.59991819448791</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.446687717335403</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-8.905512848987691</v>
+        <v>-8.905512851323831</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>426.9218052140449</v>
+        <v>426.9218052140457</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>16.25</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>49.38869974170048</v>
+        <v>49.38869980831303</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>28.0842237094229</v>
+        <v>28.08422369309777</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>1.109442433643033</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.006622878097995</v>
+        <v>-0.006622878188847381</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>53.63508549866895</v>
+        <v>53.63508552652952</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>16.24133678264</v>
+        <v>16.2413370255578</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.259450885721998</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.1859153398547704</v>
+        <v>-0.1859153395173283</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>46.00745577513332</v>
+        <v>46.00745581589143</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>26.1163426051066</v>
+        <v>26.11634265728335</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.6080589348727846</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-2.232446743315829</v>
+        <v>-2.232446744224325</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>410.8119693745644</v>
+        <v>410.8119693745645</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>67</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>52.8380686534103</v>
+        <v>52.83806868368113</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>9.290954772106545</v>
+        <v>9.290954763750749</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.6769640419266396</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1.987121058013556</v>
+        <v>1.987121058143345</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>410.1524126407031</v>
+        <v>410.152412640703</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>109</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>51.25323880523849</v>
+        <v>51.25323879625366</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>5.582416568651652</v>
+        <v>5.58241656865165</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.1625319197506941</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.9432367975048714</v>
+        <v>0.9432367977644454</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>407.9205111529605</v>
+        <v>407.9205111529589</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>32.2</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>50.06347655314166</v>
+        <v>50.06347669127023</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>14.82794157656066</v>
+        <v>14.8279416369689</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.6733904502910852</v>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>56.90480581814902</v>
+        <v>56.90480641615839</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>29.20321250171909</v>
+        <v>29.20321258190327</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.654900179788007</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.04548230960491761</v>
+        <v>-0.04548230976065681</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>40.77011785393951</v>
+        <v>40.77011798521091</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>20.57605672553709</v>
+        <v>20.57605674026334</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.4583399988051551</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-3.924670296047719</v>
+        <v>-3.924670298124319</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>44.22736917444618</v>
+        <v>44.22736912733334</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>33.39151483638064</v>
+        <v>33.39151495066193</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.3039894071370214</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-11.89726560644364</v>
+        <v>-11.89726560592455</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>43.3174910267001</v>
+        <v>43.31749103454769</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>23.7439300605601</v>
+        <v>23.74393012690111</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.5215898384106048</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-1.953476088852238</v>
+        <v>-1.953476089760776</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>396.0158340948728</v>
+        <v>396.0158340948732</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>73.5</v>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>42.40197876800653</v>
+        <v>42.40197883726679</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>26.61228889778306</v>
+        <v>26.61228900064672</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.9137828009951274</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.09846076387085176</v>
+        <v>-0.09846076420829625</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>393.4801269346866</v>
+        <v>393.4801269346872</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>269</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>47.64458922921759</v>
+        <v>47.64458926164286</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>27.92064848170981</v>
+        <v>27.92064855565813</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.7996804081804292</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-2.356640379674065</v>
+        <v>-2.356640380582544</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>392.3147385276372</v>
+        <v>392.314738527637</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>1335</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>31.13021788798123</v>
+        <v>31.13021786676531</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>20.36618884871935</v>
+        <v>20.3661888783672</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.7061025102770043</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-36.99969355375319</v>
+        <v>-36.99969355063831</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>52.55327704914463</v>
+        <v>52.55327706290964</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>6.814219190637398</v>
+        <v>6.814219210283335</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.4046173189588294</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>1.487261296254246</v>
+        <v>1.48726129560532</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>380.0704135290169</v>
+        <v>380.0704135290167</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>1380</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>25.75383666412691</v>
+        <v>25.75383667758418</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>22.33365748805273</v>
+        <v>22.3336576724544</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.6871037897598586</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-49.66011852516625</v>
+        <v>-49.66011853087697</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>46.33358604745468</v>
+        <v>46.33358595852224</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>17.99221952159467</v>
+        <v>17.99221964658617</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.5550907693913993</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.1872107654464</v>
+        <v>0.187210767263424</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>32.01575899601663</v>
+        <v>32.01575903134243</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>44.31000848339303</v>
+        <v>44.31000873252145</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>1.021781670257369</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-0.2507436375295433</v>
+        <v>-0.2507436376593286</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>362.7606918725131</v>
+        <v>362.7606918725133</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>113.5</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>42.06589688748287</v>
+        <v>42.06589707103283</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>22.81725232619706</v>
+        <v>22.81725242926304</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.3727461539875384</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-1.062866905030309</v>
+        <v>-1.062866905679234</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>46.54838514259432</v>
+        <v>46.54838537419661</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>19.54442462673784</v>
+        <v>19.54442481316146</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.531096388117119</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.8049796836688909</v>
+        <v>-0.804979686005064</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>40.51928924808804</v>
+        <v>40.51928927695452</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>16.99356758587145</v>
+        <v>16.99356760834561</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.800373782363989</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>2.064124706647391</v>
+        <v>2.064124698081343</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>344.366989852951</v>
+        <v>344.3669898529504</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>2215</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>32.89157411080305</v>
+        <v>32.8915741309428</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>16.4565856093425</v>
+        <v>16.4565857445361</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.768954451410912</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-41.39222308499306</v>
+        <v>-41.39222309381881</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>31.07772996741393</v>
+        <v>31.07772945520323</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>28.0300294681603</v>
+        <v>28.03002974364895</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.273527240156384</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-1.267688907044992</v>
+        <v>-1.267688898738662</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>27.37856116337281</v>
+        <v>27.37856119218378</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>39.28481918054652</v>
+        <v>39.28481923682392</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.347846864942765</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.01917078702889652</v>
+        <v>-0.01917078715868759</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>40.73883149925342</v>
+        <v>40.73883146254154</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>29.58451862485837</v>
+        <v>29.58451869744193</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.3134480570189231</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-13.37094748266765</v>
+        <v>-13.37094748136983</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>329.1976078372026</v>
+        <v>329.1976078372027</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>326</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>36.45233884489956</v>
+        <v>36.4523388962487</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>21.68290560790122</v>
+        <v>21.68290560785686</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.3517201685041609</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-5.525944690635571</v>
+        <v>-5.525944689597289</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>327.6742808099283</v>
+        <v>327.6742808099282</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>92.09999999999999</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>33.32899263644863</v>
+        <v>33.3289928194597</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>17.49548813118493</v>
+        <v>17.49548847186086</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.014744533036885</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.4023132657298101</v>
+        <v>-0.4023132685851163</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>46.30848977573935</v>
+        <v>46.30848974932545</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>23.57733947809583</v>
+        <v>23.57733952795464</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.4224235764427686</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-8.523146690285376</v>
+        <v>-8.523146692361863</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>36.57377918288389</v>
+        <v>36.57377924641126</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>24.4512736285377</v>
+        <v>24.45127368328428</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.5164638802058842</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-3.161404657090434</v>
+        <v>-3.161404658258529</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>319.0652754847615</v>
+        <v>319.0652754847714</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>100</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>51.40629975983297</v>
+        <v>51.40629970277309</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>11.75318057832731</v>
+        <v>11.75318079273687</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.5800087639967554</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.9574754289844147</v>
+        <v>0.9574754300227193</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>30.28557404055972</v>
+        <v>30.28557411803338</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>22.49649461164328</v>
+        <v>22.49649464205</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.7858790036747049</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-13.33695379337761</v>
+        <v>-13.33695379480525</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>40.05959334735019</v>
+        <v>40.05959352880568</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>16.78234528160664</v>
+        <v>16.78234532587113</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.3097888124258223</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-2.661332752180308</v>
+        <v>-2.661332754256875</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3824,7 +3824,7 @@
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>313.9025366551041</v>
+        <v>313.9025366551018</v>
       </c>
       <c r="E64" s="2" t="n">
         <v>25.15</v>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>46.95262209166238</v>
+        <v>46.95262217644544</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>21.8084871618374</v>
+        <v>21.80848719293608</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>1.288485978141151</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.1070551987555382</v>
+        <v>-0.1070551986257538</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>33.33559480873001</v>
+        <v>33.3355948171851</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>13.94798178538147</v>
+        <v>13.94798183698733</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.8945379952139533</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-31.0750496188203</v>
+        <v>-31.07504962297353</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.16997108707716</v>
+        <v>47.16997098763768</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>37.38035592887739</v>
+        <v>37.38035598080138</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.113171283517551</v>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>37.78207035290185</v>
+        <v>37.78207024937699</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>30.32165831048233</v>
+        <v>30.32165864604097</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4258147296895938</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-6.102755757152297</v>
+        <v>-6.102755755049746</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>52.30257338888084</v>
+        <v>52.30257340932876</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>12.37491792012946</v>
+        <v>12.37491790331273</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.5076792589835432</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.3451978322855916</v>
+        <v>0.3451978320519784</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,7 +4103,7 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>32.4435641523699</v>
+        <v>32.44356438039314</v>
       </c>
       <c r="I69" s="2" t="n">
         <v>25.78684796110294</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.04567025693906501</v>
+        <v>0.04567025592672769</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4142,7 +4142,7 @@
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>297.0396477800225</v>
+        <v>297.0396477800229</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>35.55</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>44.33367918220792</v>
+        <v>44.33367910427489</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>23.86137307906039</v>
+        <v>23.8613730724286</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.4422300185736607</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>23.72367830823855</v>
+        <v>23.72367837374966</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>38.1093283962639</v>
+        <v>38.10932845576447</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.5856268963969677</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.1529160488215631</v>
+        <v>0.1529160481726253</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>293.50014634475</v>
+        <v>293.5001463447502</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>34.75</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>43.72171927257315</v>
+        <v>43.72171791151176</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>20.99686291341275</v>
+        <v>20.99686307108684</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.4341817591629035</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.07811852851088041</v>
+        <v>-0.07811852736875824</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>46.23070701191042</v>
+        <v>46.23070697159302</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>6.836879460820192</v>
+        <v>6.836879459417654</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.5945156982702401</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.1093490150795011</v>
+        <v>0.1093490152093057</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>43.2720623198377</v>
+        <v>43.27206258107597</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>17.491288925305</v>
+        <v>17.49128883061344</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1.900130514521112</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.2628419931569761</v>
+        <v>-0.2628419940654732</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>28.1108257855909</v>
+        <v>28.11082583607896</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>30.12204594058598</v>
+        <v>30.12204606954237</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.2674659537101756</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-2.203232264523239</v>
+        <v>-2.203232265094301</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>273.6031644074378</v>
+        <v>273.6031644074389</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>144.5</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>38.28833210238486</v>
+        <v>38.28833206922826</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>10.04219783123695</v>
+        <v>10.04219779844542</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.8404747142513072</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.1416812701032244</v>
+        <v>0.1416812688053586</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>272.5342382106256</v>
+        <v>272.5342382106261</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>31.8</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>51.54385019823841</v>
+        <v>51.54384925840737</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>18.9818243914851</v>
+        <v>18.98182547174923</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.3685593678176707</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.01152541537179136</v>
+        <v>-0.01152541464498685</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>272.4957578906539</v>
+        <v>272.4957578906536</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>456</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>35.65039149289042</v>
+        <v>35.65039155177837</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>27.88087010880307</v>
+        <v>27.88087014027306</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>1.345583126836235</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-7.025422158947936</v>
+        <v>-7.025422157650122</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>272.4562513076618</v>
+        <v>272.4562513076623</v>
       </c>
       <c r="E79" s="2" t="n">
         <v>18.2</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>40.01732771759666</v>
+        <v>40.01732770050351</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>25.44620951193615</v>
+        <v>25.44620946498283</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.6849304406437724</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.0752232845104423</v>
+        <v>-0.07522328449746499</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>271.0990234080965</v>
+        <v>271.0990234080953</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>90.8</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>45.9108220666081</v>
+        <v>45.91082362436342</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.58637067314796</v>
+        <v>14.58637074408145</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.8406476273621756</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.05471678122270274</v>
+        <v>-0.05471678252057499</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>44.5788779214393</v>
+        <v>44.57887834779962</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>15.11538527686319</v>
+        <v>15.11538545079234</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.2192994479136399</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.07986155068320386</v>
+        <v>0.07986154993044095</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>39.98389624678777</v>
+        <v>39.98389497255923</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>21.26953979735394</v>
+        <v>21.26954049110333</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.654961637642864</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.4375885978306194</v>
+        <v>-0.4375885948455238</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4831,7 +4831,7 @@
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>265.3984907439227</v>
+        <v>265.3984907439221</v>
       </c>
       <c r="E83" s="2" t="n">
         <v>58.9</v>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>54.00663905701465</v>
+        <v>54.00663936150787</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>19.20475935030805</v>
+        <v>19.2047594166101</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.441339772438632</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.5480401412092448</v>
+        <v>-0.5480401431560469</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>261.0596499352913</v>
+        <v>261.0596499352912</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>29</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>28.81826737526406</v>
+        <v>28.81826696791758</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>15.99904749867302</v>
+        <v>15.99904783551976</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>2.034100240657322</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.04566869235165275</v>
+        <v>-0.04566869222187123</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>30.02768145936381</v>
+        <v>30.02768147830079</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>20.12689927126038</v>
+        <v>20.12689925992729</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.633601876040858</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-1.314608430550331</v>
+        <v>-1.314608431199294</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>249.8894856464012</v>
+        <v>249.8894856464008</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>767</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>28.78813061589571</v>
+        <v>28.78813062931786</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>21.55837039189321</v>
+        <v>21.55837023068175</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.7436915778798949</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-19.1835292659071</v>
+        <v>-19.18352927161774</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>36.34703708546677</v>
+        <v>36.34703708890324</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>18.82816872651384</v>
+        <v>18.82816875683433</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.4541186164436287</v>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>51.38197040929622</v>
+        <v>51.38197039376421</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>13.77828059894971</v>
+        <v>13.77828058098923</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>1.369059722541078</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-3.041457934696523</v>
+        <v>-3.0414579359944</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>25.94153879879708</v>
+        <v>25.94153887234572</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>46.64211308354098</v>
+        <v>46.64211318546129</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.3560207270805228</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>29.0633107347394</v>
+        <v>29.06331072917862</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>33.09182901892147</v>
+        <v>33.09182977897751</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>34.15273231116273</v>
+        <v>34.15273242136041</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.8016316280463053</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.307059097243032</v>
+        <v>0.3070590994493951</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>238.7465675666309</v>
+        <v>238.7465675666339</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>48.8</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>41.16776853891192</v>
+        <v>41.1677686455759</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>23.36267676678313</v>
+        <v>23.36267682486515</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.3843941879937076</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.01883653935127449</v>
+        <v>-0.01883653945510405</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>29.21128879538763</v>
+        <v>29.21128933378034</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>16.24140452435922</v>
+        <v>16.24140465471655</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.320137439706831</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.008299979102753707</v>
+        <v>0.00829997886914241</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>44.55876189037313</v>
+        <v>44.55876170393005</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>22.31929775997412</v>
+        <v>22.31929782844946</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.122901913826207</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>41.20542922899121</v>
+        <v>41.20542968085091</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>17.96371292411992</v>
+        <v>17.96371302502378</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.4672757876682647</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.9005407598628175</v>
+        <v>0.9005407599926061</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>38.82198883945414</v>
+        <v>38.82198876670596</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>35.14721052732221</v>
+        <v>35.14721048556191</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.08875215532512933</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.3899324410505247</v>
+        <v>0.3899324412841487</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>44.94797147410826</v>
+        <v>44.94797150867501</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>18.79521160600477</v>
+        <v>18.79521155537881</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.3850648513387129</v>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>48.89003571146712</v>
+        <v>48.89003582284947</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>27.26238295275843</v>
+        <v>27.26238299194468</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.6009768353449475</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.07098613541194887</v>
+        <v>-0.07098613543790638</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>32.62910746490004</v>
+        <v>32.62910705625453</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>29.33231825791877</v>
+        <v>29.33231853319658</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.3224629159536419</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-3.008824421799343</v>
+        <v>-3.00882441868445</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>43.38767217474861</v>
+        <v>43.38767219479106</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>15.7140944655928</v>
+        <v>15.71409453740554</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.4966433622443178</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-4.779138284014996</v>
+        <v>-4.779138284534186</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5838,7 +5838,7 @@
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>209.8887574599575</v>
+        <v>209.8887574599574</v>
       </c>
       <c r="E102" s="2" t="n">
         <v>27.5</v>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>31.7532174561822</v>
+        <v>31.75321766518717</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>14.19190151986884</v>
+        <v>14.19190159849589</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.5419144607278206</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.2074825913339464</v>
+        <v>-0.2074825922294758</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>38.97660836067052</v>
+        <v>38.97660878914031</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>20.17450748321274</v>
+        <v>20.17450746992235</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>2.195539622104401</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-1.693580999141405</v>
+        <v>-1.693581003164804</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>40.50354334420683</v>
+        <v>40.50354333426358</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>13.41129180542102</v>
+        <v>13.41129181608641</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.6354606498296433</v>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>201.489761172531</v>
+        <v>201.4897611725307</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>324.5</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>31.88568361878951</v>
+        <v>31.88568377333236</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>25.25398597015161</v>
+        <v>25.25398593784459</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.4577428042906045</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-5.993471076272529</v>
+        <v>-5.993471083281037</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>197.0847663499844</v>
+        <v>197.0847663499845</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>149.5</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>33.94067965821017</v>
+        <v>33.94067960907088</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>18.04612313812876</v>
+        <v>18.04612327704535</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.7281824407457832</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-2.166772782507923</v>
+        <v>-2.166772782378142</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>34.3624746050575</v>
+        <v>34.36247466014487</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>20.88417812920435</v>
+        <v>20.88417823996821</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>1.466730410043331</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.2897840605544456</v>
+        <v>-0.2897840609178541</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>188.0490843707243</v>
+        <v>188.0490843707242</v>
       </c>
       <c r="E108" s="2" t="n">
         <v>11.9</v>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>34.74831139306306</v>
+        <v>34.74831130601521</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>21.81628554915564</v>
+        <v>21.81628540355981</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.7163049738704035</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.03220424678541584</v>
+        <v>-0.03220424679839326</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>187.1922876878696</v>
+        <v>187.1922876878693</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>159.5</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>32.57627477214706</v>
+        <v>32.57627481057601</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>26.32959228199431</v>
+        <v>26.32959242719334</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.9406997937471052</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.3750262667293813</v>
+        <v>-0.375026267248503</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>25.70969764544633</v>
+        <v>25.7096989031707</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>21.38305562017104</v>
+        <v>21.38305557279875</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>1.016609847516595</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.1443610440437436</v>
+        <v>-0.1443610446926757</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>183.7599490124171</v>
+        <v>183.7599490124176</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>15.05</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>25.6428394107392</v>
+        <v>25.64283898898245</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>20.64747900698251</v>
+        <v>20.64747947396137</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>1.729007181179986</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.1236964166495151</v>
+        <v>-0.1236964163250469</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>39.25566945734047</v>
+        <v>39.25566949276527</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>17.85990100310328</v>
+        <v>17.85990102904315</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.9526613838198412</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.223992477381264</v>
+        <v>0.2239924766025558</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>35.45025736054042</v>
+        <v>35.45025766256286</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>29.96303962712103</v>
+        <v>29.96303996000574</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.3175174391228578</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.03792028777664935</v>
+        <v>0.03792028767282385</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>175.5732874389897</v>
+        <v>175.5732874389874</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>136</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>44.43983885089376</v>
+        <v>44.43983864191284</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>17.90093401062109</v>
+        <v>17.90093397741712</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.9943424826983293</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.6450103209124199</v>
+        <v>-0.6450103203932613</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>39.87702616852852</v>
+        <v>39.87702634945363</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>26.92587813333784</v>
+        <v>26.9258781903117</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.563655617073422</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.06877389208792328</v>
+        <v>-0.06877389278876844</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>28.11688283876856</v>
+        <v>28.11688305536011</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>11.3079333175439</v>
+        <v>11.30793333597864</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.7685597441157561</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.2227020187905615</v>
+        <v>-0.2227020186607662</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6633,7 +6633,7 @@
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>163.3595488511895</v>
+        <v>163.3595488511899</v>
       </c>
       <c r="E117" s="2" t="n">
         <v>57.4</v>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>20.59360609539162</v>
+        <v>20.5936061652221</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>14.49182788256149</v>
+        <v>14.49182781319054</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>4.021508906430247</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.4487798883035834</v>
+        <v>-0.4487798890823038</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>39.3688141052918</v>
+        <v>39.36881415833792</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>17.25639947586482</v>
+        <v>17.25639960495843</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.6644970316679577</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-2.183333645812937</v>
+        <v>-2.183333647889537</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>51.47476530270618</v>
+        <v>51.47476529479479</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>4.786972665000263</v>
+        <v>4.786972709018599</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>1.084288657354927</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.160033934268681</v>
+        <v>0.1600339341388994</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>129.1091885705272</v>
+        <v>129.1091885705276</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>15.65</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>37.02072110963681</v>
+        <v>37.02074664601204</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.23203251719088</v>
+        <v>15.23202572308351</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.8373586176754699</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.02321817194183362</v>
+        <v>-0.02321817770858725</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>122.5825622446062</v>
+        <v>122.5825622446082</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>25.3</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>26.14012147089841</v>
+        <v>26.14012148714799</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>24.16427851622451</v>
+        <v>24.16427861038929</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.2915990655167355</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.04248755097985191</v>
+        <v>-0.04248755113559421</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>120.3509562514848</v>
+        <v>120.350956251485</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>249</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>31.52889846460468</v>
+        <v>31.52889863935657</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>14.09416570981813</v>
+        <v>14.09416564606516</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>1.25176317180764</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.6847255914093111</v>
+        <v>-0.6847255947837869</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>39.19665909680835</v>
+        <v>39.1966593272096</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.17440670224569</v>
+        <v>13.17440692386337</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>1.092703328027108</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.223357282063857</v>
+        <v>-0.2233572824532173</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>108.1222171030566</v>
+        <v>108.1222171030564</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>265.5</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>37.28549049568746</v>
+        <v>37.2854904236905</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>17.36300252499322</v>
+        <v>17.36300254019361</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.4677438334097521</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-3.929460935124947</v>
+        <v>-3.929460933697228</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>108.0471407190916</v>
+        <v>108.0471407190917</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>547</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>34.54311408569345</v>
+        <v>34.54311418470519</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>18.74096187510991</v>
+        <v>18.7409619506133</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.2637643471107782</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-8.921718140067426</v>
+        <v>-8.921718145648235</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>100.1426058692759</v>
+        <v>100.1426058692707</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>16.75</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>43.5002553964326</v>
+        <v>43.50025562478501</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>19.65312678005457</v>
+        <v>19.65312675709144</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.1888328657471896</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.01633143812894894</v>
+        <v>-0.01633143832362741</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7163,7 +7163,7 @@
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>97.74219917463161</v>
+        <v>97.74219917463159</v>
       </c>
       <c r="E127" s="2" t="n">
         <v>24.5</v>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>20.13595955367859</v>
+        <v>20.1359595935498</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>16.93497544303577</v>
+        <v>16.93497553835291</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.6002778183225612</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.03347239783865352</v>
+        <v>-0.03347239843567795</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>45.73796484467013</v>
+        <v>45.73796497625422</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>17.22361051080645</v>
+        <v>17.22361057253819</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.4034722290199748</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>-0.2111764715112427</v>
+        <v>-0.2111764719525156</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg7 2026-10-27 00:08 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-10-22.xlsx
+++ b/output/full_scan/batch_seq8_2026-10-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>69.94965175462735</v>
+        <v>69.9496517463252</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>19.19329802336328</v>
+        <v>19.19329804291291</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>7.940162131896488</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>0.3163592924948281</v>
+        <v>0.3163592926209806</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>68.03869779931199</v>
+        <v>68.03869786058718</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>21.28026604239151</v>
+        <v>21.28026606677422</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>2.504310862823595</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1.052771918549143</v>
+        <v>1.052771917960438</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>74.45730782053397</v>
+        <v>74.45730781340255</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>39.0104089987615</v>
+        <v>39.01040901680027</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.722705245415632</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>3.463566899436183</v>
+        <v>3.463566899996847</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>59.33528986086874</v>
+        <v>59.33528995501849</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>24.76698919142567</v>
+        <v>24.76698920609061</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>7.622238109654431</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>1.163103766354558</v>
+        <v>1.163103766074213</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>70.83526072578613</v>
+        <v>70.83526063403102</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>52.3362311663102</v>
+        <v>52.33623151205342</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>4.641489785575262</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>3.030560989834909</v>
+        <v>3.030560990255418</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>62.1859254895444</v>
+        <v>62.18592544488873</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>29.19834311325341</v>
+        <v>29.19834317791531</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.217630350492084</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.710352958835055</v>
+        <v>1.710352961077811</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>783.1688664672783</v>
+        <v>783.1688664672788</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>420</v>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>64.3003150505638</v>
+        <v>64.30031515313107</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>37.03299660972345</v>
+        <v>37.03299690725727</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>1.604068862259369</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>5.203575770439357</v>
+        <v>5.203575767495821</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>67.34293755549697</v>
+        <v>67.34293752751745</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>62.76794308880867</v>
+        <v>62.76794307478276</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.6413756187117383</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>-2.67697981547127</v>
+        <v>-2.676979813929371</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>54.7248016368945</v>
+        <v>54.72480171133832</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>26.9003311091649</v>
+        <v>26.90033111800057</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>2.150892226377595</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-5.85393457660328</v>
+        <v>-5.853934580107495</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>53.19198551361392</v>
+        <v>53.19198559292669</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>24.06601552382029</v>
+        <v>24.06601549425053</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.34306299199178</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.6402986371487178</v>
+        <v>-0.640298637849567</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>56.31363707311227</v>
+        <v>56.3136370608814</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>32.75928343774675</v>
+        <v>32.7592834341166</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>1.042011461143822</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.6696098661538343</v>
+        <v>-0.6696098662098979</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>631.352816169261</v>
+        <v>631.3528161692608</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>24.95</v>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>57.47428873134015</v>
+        <v>57.47429022479751</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>17.20984192539955</v>
+        <v>17.20984221782384</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.691032403918613</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.1692508146734619</v>
+        <v>0.169250814210907</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>52.53769618541418</v>
+        <v>52.53769621843419</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>18.42807184930868</v>
+        <v>18.42807201227319</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.9261545656685027</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.4446222571126914</v>
+        <v>0.4446222569725338</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         <v>63.5727237145042</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>27.71466386217883</v>
+        <v>27.71466392617614</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.895021888780528</v>
@@ -1294,7 +1294,7 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>56.92213959713399</v>
+        <v>56.92213962005316</v>
       </c>
       <c r="I16" s="2" t="n">
         <v>29.3251052955181</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.838892873662398</v>
+        <v>0.8388928733540206</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>52.74685587979288</v>
+        <v>52.74685587154042</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>46.44135771463289</v>
+        <v>46.44135772045016</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.6281562191566618</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>-5.226515709525671</v>
+        <v>-5.226515708964982</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1386,7 @@
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>587.3927484592128</v>
+        <v>587.3927484592125</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>5275</v>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>40.83948143861321</v>
+        <v>40.83948143650147</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>14.26846172783942</v>
+        <v>14.2684616567777</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.010550192051703</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>-55.80704447964263</v>
+        <v>-55.8070444782403</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>50.57197283127809</v>
+        <v>50.57197250760128</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>40.24573200609252</v>
+        <v>40.24573206799976</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.3216410277318243</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>-0.3599697687560817</v>
+        <v>-0.3599697683355734</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>482.8926257339058</v>
+        <v>482.8926257339059</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>119</v>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>51.09637824097655</v>
+        <v>51.09637854740167</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>16.90952776231768</v>
+        <v>16.90952775152432</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>1.030996144758115</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.4254610190147214</v>
+        <v>0.4254610188745623</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>476.3138932595559</v>
+        <v>476.3138932595547</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>45.9</v>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>49.20573112498275</v>
+        <v>49.20573217420865</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>12.52309821182338</v>
+        <v>12.52309828788268</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>0.5902387289890044</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.2250852720962755</v>
+        <v>0.2250852713393497</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>37.91715399898477</v>
+        <v>37.9171544222876</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>13.56403198373947</v>
+        <v>13.56403201085486</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.6650754418188766</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-0.6837150996380408</v>
+        <v>-0.683715099918365</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>43.19175202554241</v>
+        <v>43.19175179895286</v>
       </c>
       <c r="I25" s="2" t="n">
         <v>27.17915790035438</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.1576494230550256</v>
+        <v>-0.1576494226345242</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>459.6270241187337</v>
+        <v>459.6270241187326</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>48.5</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>58.01707416274689</v>
+        <v>58.01707412958065</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>39.61825314176064</v>
+        <v>39.61825322836825</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>3.122163418376172</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.5196112413479834</v>
+        <v>0.5196112412498628</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>449.4834192354285</v>
+        <v>449.4834192354286</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>39.2</v>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>52.19316830289503</v>
+        <v>52.193168293283</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>6.517310348231315</v>
+        <v>6.517310218353303</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.5330006106749495</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.08312193232785448</v>
+        <v>0.08312193235588605</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>44.26001799550453</v>
+        <v>44.26001799737104</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>25.43737028424433</v>
+        <v>25.43737028538833</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.2126352000985455</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-6.459398176540606</v>
+        <v>-6.459398176680791</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>35.53863552284471</v>
+        <v>35.53863554213814</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>21.62935468199205</v>
+        <v>21.62935474289196</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.6702648318182373</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>-3.20546224073101</v>
+        <v>-3.205462241291667</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>45.37340792240466</v>
+        <v>45.37340793476122</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>19.59991819448791</v>
+        <v>19.59991842415261</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>1.446687717335403</v>
@@ -2075,7 +2075,7 @@
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>426.9218052140457</v>
+        <v>426.9218052140455</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>16.25</v>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>49.38869980831303</v>
+        <v>49.38869991724977</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>28.08422369309777</v>
+        <v>28.08422359981473</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>1.109442433643033</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.006622878188847381</v>
+        <v>-0.006622878230898938</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>424.1353704579694</v>
+        <v>424.1353704579701</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>40.3</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>53.63508552652952</v>
+        <v>53.63508539901382</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>16.2413370255578</v>
+        <v>16.24133729698649</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>1.259450885721998</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.1859153395173283</v>
+        <v>-0.1859153390407454</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>46.00745581589143</v>
+        <v>46.00745582320699</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>26.11634265728335</v>
+        <v>26.11634265310756</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>0.6080589348727846</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-2.232446744224325</v>
+        <v>-2.232446744364498</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>410.8119693745645</v>
+        <v>410.8119693745646</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>67</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>52.83806868368113</v>
+        <v>52.83806864353571</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>9.290954763750749</v>
+        <v>9.29095461675052</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>0.6769640419266396</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>1.987121058143345</v>
+        <v>1.987121060245891</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>410.152412640703</v>
+        <v>410.1524126407031</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>109</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>51.25323879625366</v>
+        <v>51.25323880357127</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>5.58241656865165</v>
+        <v>5.582416700160416</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.1625319197506941</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.9432367977644454</v>
+        <v>0.9432367974840918</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>407.9205111529589</v>
+        <v>407.9205111529582</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>32.2</v>
@@ -2354,7 +2354,7 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>50.06347669127023</v>
+        <v>50.06347644309501</v>
       </c>
       <c r="I36" s="2" t="n">
         <v>14.8279416369689</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.002686765335479541</v>
+        <v>0.002686765419586262</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>56.90480641615839</v>
+        <v>56.90480577214831</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>29.20321258190327</v>
+        <v>29.2032126296392</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>0.654900179788007</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.04548230976065681</v>
+        <v>-0.04548230936818365</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>40.77011798521091</v>
+        <v>40.7701181019262</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>20.57605674026334</v>
+        <v>20.57605675197868</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.4583399988051551</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-3.924670298124319</v>
+        <v>-3.924670296442263</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,7 +2513,7 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>44.22736912733334</v>
+        <v>44.22736917487823</v>
       </c>
       <c r="I39" s="2" t="n">
         <v>33.39151495066193</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-11.89726560592455</v>
+        <v>-11.89726560802707</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>43.31749103454769</v>
+        <v>43.31749108332278</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>23.74393012690111</v>
+        <v>23.7439302196394</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.5215898384106048</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-1.953476089760776</v>
+        <v>-1.953476090461608</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>396.0158340948732</v>
+        <v>396.0158340948733</v>
       </c>
       <c r="E41" s="2" t="n">
         <v>73.5</v>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>42.40197883726679</v>
+        <v>42.40197894462172</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>26.61228900064672</v>
+        <v>26.61228910219113</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.9137828009951274</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.09846076420829625</v>
+        <v>-0.09846076437650564</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>393.4801269346872</v>
+        <v>393.4801269346864</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>269</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>47.64458926164286</v>
+        <v>47.64458922672335</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>27.92064855565813</v>
+        <v>27.92064849113815</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.7996804081804292</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-2.356640380582544</v>
+        <v>-2.356640380862903</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>392.314738527637</v>
+        <v>392.3147385276372</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>1335</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>31.13021786676531</v>
+        <v>31.13021787223907</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>20.3661888783672</v>
+        <v>20.36618889628118</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.7061025102770043</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-36.99969355063831</v>
+        <v>-36.99969355175959</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>52.55327706290964</v>
+        <v>52.5532770598013</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>6.814219210283335</v>
+        <v>6.814219249766968</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>0.4046173189588294</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>1.48726129560532</v>
+        <v>1.487261296166006</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>380.0704135290167</v>
+        <v>380.0704135290169</v>
       </c>
       <c r="E45" s="2" t="n">
         <v>1380</v>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>25.75383667758418</v>
+        <v>25.75383668666595</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>22.3336576724544</v>
+        <v>22.33365767128499</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.6871037897598586</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-49.66011853087697</v>
+        <v>-49.66011853101732</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>365.5619634847518</v>
+        <v>365.5619634847515</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>131.5</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>46.33358595852224</v>
+        <v>46.33358598588607</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>17.99221964658617</v>
+        <v>17.99221973646166</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>0.5550907693913993</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.187210767263424</v>
+        <v>0.1872107682446188</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>363.3842911122858</v>
+        <v>363.3842911122859</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>50.3</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>32.01575903134243</v>
+        <v>32.01575884112665</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>44.31000873252145</v>
+        <v>44.31000860869823</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>1.021781670257369</v>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>362.7606918725133</v>
+        <v>362.7606918725132</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>113.5</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>42.06589707103283</v>
+        <v>42.0658968950102</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>22.81725242926304</v>
+        <v>22.81725273646522</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.3727461539875384</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-1.062866905679234</v>
+        <v>-1.062866905258721</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>46.54838537419661</v>
+        <v>46.54838525888408</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>19.54442481316146</v>
+        <v>19.54442483974081</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.531096388117119</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.804979686005064</v>
+        <v>-0.8049796850238566</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>354.6869061881474</v>
+        <v>354.6869061881475</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>1810</v>
@@ -3149,7 +3149,7 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>40.51928927695452</v>
+        <v>40.5192892665922</v>
       </c>
       <c r="I51" s="2" t="n">
         <v>16.99356760834561</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>2.064124698081343</v>
+        <v>2.064124697240388</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>344.3669898529504</v>
+        <v>344.3669898529506</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>2215</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>32.8915741309428</v>
+        <v>32.89157412674446</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>16.4565857445361</v>
+        <v>16.4565857669705</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.768954451410912</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-41.39222309381881</v>
+        <v>-41.39222309269746</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>31.07772945520323</v>
+        <v>31.07772992444959</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>28.03002974364895</v>
+        <v>28.03002974364894</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>1.273527240156384</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>-1.267688898738662</v>
+        <v>-1.267688907989871</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3294,7 @@
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>331.5917558074496</v>
+        <v>331.5917558074495</v>
       </c>
       <c r="E54" s="2" t="n">
         <v>67.40000000000001</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>27.37856119218378</v>
+        <v>27.37856120769737</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>39.28481923682392</v>
+        <v>39.2848192441138</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>1.347846864942765</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.01917078715868759</v>
+        <v>-0.01917078724279708</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>40.73883146254154</v>
+        <v>40.7388315578937</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>29.58451869744193</v>
+        <v>29.58451875449528</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.3134480570189231</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-13.37094748136983</v>
+        <v>-13.37094748193046</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>36.4523388962487</v>
+        <v>36.45233884094963</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>21.68290560785686</v>
+        <v>21.68290574077886</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.3517201685041609</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-5.525944689597289</v>
+        <v>-5.525944687354596</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>33.3289928194597</v>
+        <v>33.32899370650067</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>17.49548847186086</v>
+        <v>17.49548875784623</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.014744533036885</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-0.4023132685851163</v>
+        <v>-0.4023132699868159</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>327.3682340634665</v>
+        <v>327.3682340634664</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>759</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>46.30848974932545</v>
+        <v>46.30848978843834</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>23.57733952795464</v>
+        <v>23.57733961074531</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.4224235764427686</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-8.523146692361863</v>
+        <v>-8.523146696847478</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>36.57377924641126</v>
+        <v>36.57377933483421</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>24.45127368328428</v>
+        <v>24.45127367855582</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>0.5164638802058842</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-3.161404658258529</v>
+        <v>-3.161404658118358</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>319.0652754847714</v>
+        <v>319.0652754847619</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>100</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>51.40629970277309</v>
+        <v>51.40629975466891</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>11.75318079273687</v>
+        <v>11.75318073662445</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.5800087639967554</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.9574754300227193</v>
+        <v>0.9574754251167725</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>30.28557411803338</v>
+        <v>30.28557404136778</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>22.49649464205</v>
+        <v>22.49649462389461</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.7858790036747049</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-13.33695379480525</v>
+        <v>-13.33695379172157</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>40.05959352880568</v>
+        <v>40.05959351888276</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>16.78234532587113</v>
+        <v>16.78234527140389</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.3097888124258223</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-2.661332754256875</v>
+        <v>-2.661332752995354</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>46.95262217644544</v>
+        <v>46.95262182521308</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>21.80848719293608</v>
+        <v>21.80848737818291</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>1.288485978141151</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.1070551986257538</v>
+        <v>-0.1070551984014795</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>33.3355948171851</v>
+        <v>33.33559480216105</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>13.94798183698733</v>
+        <v>13.94798188608963</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.8945379952139533</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-31.07504962297353</v>
+        <v>-31.07504962465531</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>47.16997098763768</v>
+        <v>47.16997109472636</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>37.38035598080138</v>
+        <v>37.38035597844277</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.113171283517551</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.0189572876883817</v>
+        <v>-0.01895728780051659</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>37.78207024937699</v>
+        <v>37.782070169268</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>30.32165864604097</v>
+        <v>30.32165896977111</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>0.4258147296895938</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-6.102755755049746</v>
+        <v>-6.102755755133841</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>52.30257340932876</v>
+        <v>52.30257342494805</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>12.37491790331273</v>
+        <v>12.37491813161003</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.5076792589835432</v>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>301.2664344223953</v>
+        <v>301.2664344223954</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>62.3</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>32.44356438039314</v>
+        <v>32.44356420871698</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>25.78684796110294</v>
+        <v>25.78684841714903</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.8055356475983216</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.04567025592672769</v>
+        <v>0.04567025620706255</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4142,7 +4142,7 @@
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>297.0396477800229</v>
+        <v>297.0396477800254</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>35.55</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>44.33367910427489</v>
+        <v>44.33367936383888</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>23.8613730724286</v>
+        <v>23.86137316129496</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.4422300185736607</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.1923270133319481</v>
+        <v>-0.1923270135842584</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>296.6897522524122</v>
+        <v>296.6897522524121</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>114.5</v>
@@ -4212,7 +4212,7 @@
         <v>23.72367837374966</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>38.10932845576447</v>
+        <v>38.10932848350232</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.5856268963969677</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.1529160481726253</v>
+        <v>0.1529160478922793</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>293.5001463447502</v>
+        <v>293.5001463447497</v>
       </c>
       <c r="E72" s="2" t="n">
         <v>34.75</v>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>43.72171791151176</v>
+        <v>43.7217185226438</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>20.99686307108684</v>
+        <v>20.99686328244071</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.4341817591629035</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.07811852736875824</v>
+        <v>-0.07811852850413228</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>46.23070697159302</v>
+        <v>46.23070706391565</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>6.836879459417654</v>
+        <v>6.836879453733492</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.5945156982702401</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.1093490152093057</v>
+        <v>0.1093490146486236</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>43.27206258107597</v>
+        <v>43.27206240267361</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>17.49128883061344</v>
+        <v>17.49128870554977</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>1.900130514521112</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.2628419940654732</v>
+        <v>-0.262841993644972</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>28.11082583607896</v>
+        <v>28.11082585872758</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>30.12204606954237</v>
+        <v>30.12204601270236</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.2674659537101756</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-2.203232265094301</v>
+        <v>-2.203232265066271</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>273.6031644074389</v>
+        <v>273.6031644074394</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>144.5</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>38.28833206922826</v>
+        <v>38.28833224314285</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>10.04219779844542</v>
+        <v>10.04219795474932</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.8404747142513072</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.1416812688053586</v>
+        <v>0.1416812669831597</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>272.5342382106261</v>
+        <v>272.5342382106253</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>31.8</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>51.54384925840737</v>
+        <v>51.54384979841279</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>18.98182547174923</v>
+        <v>18.98182553727758</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.3685593678176707</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.01152541464498685</v>
+        <v>-0.01152541509352739</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4566,7 +4566,7 @@
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>272.4957578906536</v>
+        <v>272.4957578906538</v>
       </c>
       <c r="E78" s="2" t="n">
         <v>456</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>35.65039155177837</v>
+        <v>35.6503914443327</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>27.88087014027306</v>
+        <v>27.88087007304125</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>1.345583126836235</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-7.025422157650122</v>
+        <v>-7.025422154005634</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>40.01732770050351</v>
+        <v>40.0173277189115</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>25.44620946498283</v>
+        <v>25.44620956231743</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.6849304406437724</v>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>271.0990234080953</v>
+        <v>271.0990234080966</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>90.8</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>45.91082362436342</v>
+        <v>45.91082208406675</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.58637074408145</v>
+        <v>14.58637078719614</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.8406476273621756</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.05471678252057499</v>
+        <v>-0.0547167778949853</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>44.57887834779962</v>
+        <v>44.57887864004504</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>15.11538545079234</v>
+        <v>15.11538546612726</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.2192994479136399</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.07986154993044095</v>
+        <v>0.07986154967813566</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>39.98389497255923</v>
+        <v>39.98389534938849</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>21.26954049110333</v>
+        <v>21.26954069049588</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>0.654961637642864</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.4375885948455238</v>
+        <v>-0.4375885963873858</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>54.00663936150787</v>
+        <v>54.00663939429944</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>19.2047594166101</v>
+        <v>19.20475948957307</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.441339772438632</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-0.5480401431560469</v>
+        <v>-0.548040143856894</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>261.0596499352912</v>
+        <v>261.0596499352913</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>29</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>28.81826696791758</v>
+        <v>28.81826712252362</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>15.99904783551976</v>
+        <v>15.99904781490457</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>2.034100240657322</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.04566869222187123</v>
+        <v>-0.04566869224989903</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>30.02768147830079</v>
+        <v>30.02768174650411</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>20.12689925992729</v>
+        <v>20.1268994069821</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.633601876040858</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-1.314608431199294</v>
+        <v>-1.314608431619799</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>249.8894856464008</v>
+        <v>249.8894856464011</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>767</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>28.78813062931786</v>
+        <v>28.78813062518796</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>21.55837023068175</v>
+        <v>21.55837030496154</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.7436915778798949</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-19.18352927161774</v>
+        <v>-19.1835292758228</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>36.34703708890324</v>
+        <v>36.34703708520242</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>18.82816875683433</v>
+        <v>18.8281687996443</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.4541186164436287</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.9397623443529191</v>
+        <v>-0.9397623443226388</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>51.38197039376421</v>
+        <v>51.38197041941193</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>13.77828058098923</v>
+        <v>13.77828056472997</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>1.369059722541078</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-3.0414579359944</v>
+        <v>-3.041457939498637</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>25.94153887234572</v>
+        <v>25.94153897287964</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>46.64211318546129</v>
+        <v>46.64211335919732</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.3560207270805228</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>29.06331072917862</v>
+        <v>29.06331073086015</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>33.09182977897751</v>
+        <v>33.09182990994101</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>34.15273242136041</v>
+        <v>34.1527328893314</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.8016316280463053</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.3070590994493951</v>
+        <v>0.307059105336533</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>238.7465675666339</v>
+        <v>238.7465675666309</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>48.8</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>41.1677686455759</v>
+        <v>41.16776857302312</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>23.36267682486515</v>
+        <v>23.36267705076832</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.3843941879937076</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.01883653945510405</v>
+        <v>-0.01883653942707497</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>232.4531974199631</v>
+        <v>232.4531974199635</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>37.5</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>29.21128933378034</v>
+        <v>29.21128923478547</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>16.24140465471655</v>
+        <v>16.24140463859664</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>1.320137439706831</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.00829997886914241</v>
+        <v>0.00829997909340463</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>230.0491366450005</v>
+        <v>230.0491366450004</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>43.4</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>44.55876170393005</v>
+        <v>44.55876180432247</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>22.31929782844946</v>
+        <v>22.31929765314859</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>1.122901913826207</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.0001083794905354374</v>
+        <v>-0.0001083797708770207</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>228.7641351604814</v>
+        <v>228.7641351604813</v>
       </c>
       <c r="E96" s="2" t="n">
         <v>104</v>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>41.20542968085091</v>
+        <v>41.20542897441274</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>17.96371302502378</v>
+        <v>17.96371343523657</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.4672757876682647</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.9005407599926061</v>
+        <v>0.9005407658797431</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>38.82198876670596</v>
+        <v>38.82198885484319</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>35.14721048556191</v>
+        <v>35.14721054444239</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.08875215532512933</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.3899324412841487</v>
+        <v>0.3899324413121827</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>44.94797150867501</v>
+        <v>44.94797134987549</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>18.79521155537881</v>
+        <v>18.79521144203873</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.3850648513387129</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.04829235972736842</v>
+        <v>-0.04829235969933549</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>48.89003582284947</v>
+        <v>48.89003570289925</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>27.26238299194468</v>
+        <v>27.26238337442603</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.6009768353449475</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.07098613543790638</v>
+        <v>-0.07098613529773612</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>32.62910705625453</v>
+        <v>32.62910715493318</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>29.33231853319658</v>
+        <v>29.33231871386847</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.3224629159536419</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-3.00882441868445</v>
+        <v>-3.008824419945964</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>43.38767219479106</v>
+        <v>43.38767220902487</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>15.71409453740554</v>
+        <v>15.71409452004609</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.4966433622443178</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-4.779138284534186</v>
+        <v>-4.779138284113658</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>31.75321766518717</v>
+        <v>31.75321769570679</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>14.19190159849589</v>
+        <v>14.19190164907789</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.5419144607278206</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.2074825922294758</v>
+        <v>-0.2074825923696415</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>38.97660878914031</v>
+        <v>38.97660948592457</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>20.17450746992235</v>
+        <v>20.17450745300084</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>2.195539622104401</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-1.693581003164804</v>
+        <v>-1.693581001763108</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5961,7 +5961,7 @@
         <v>40.50354333426358</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>13.41129181608641</v>
+        <v>13.41129176353905</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.6354606498296433</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.008283431795362839</v>
+        <v>-0.008283431823403187</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>201.4897611725307</v>
+        <v>201.4897611725306</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>324.5</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>31.88568377333236</v>
+        <v>31.88568372007452</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>25.25398593784459</v>
+        <v>25.2539859517218</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.4577428042906045</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-5.993471083281037</v>
+        <v>-5.993471083841715</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>197.0847663499845</v>
+        <v>197.0847663499843</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>149.5</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>33.94067960907088</v>
+        <v>33.94067962052047</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>18.04612327704535</v>
+        <v>18.04612322822318</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.7281824407457832</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-2.166772782378142</v>
+        <v>-2.166772782882747</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6103,7 +6103,7 @@
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>192.4843326960706</v>
+        <v>192.4843326960743</v>
       </c>
       <c r="E107" s="2" t="n">
         <v>58.2</v>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>34.36247466014487</v>
+        <v>34.36247555453433</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>20.88417823996821</v>
+        <v>20.88417825979419</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>1.466730410043331</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.2897840609178541</v>
+        <v>-0.2897840610860549</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>34.74831130601521</v>
+        <v>34.74831150340087</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>21.81628540355981</v>
+        <v>21.81628538604084</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.7163049738704035</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.03220424679839326</v>
+        <v>-0.03220424689651397</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>187.1922876878693</v>
+        <v>187.1922876878704</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>159.5</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>32.57627481057601</v>
+        <v>32.57627513844062</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>26.32959242719334</v>
+        <v>26.32959241875203</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.9406997937471052</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.375026267248503</v>
+        <v>-0.3750262673886944</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>25.7096989031707</v>
+        <v>25.70969773060844</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>21.38305557279875</v>
+        <v>21.38305599282037</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>1.016609847516595</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.1443610446926757</v>
+        <v>-0.1443610438516563</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>183.7599490124176</v>
+        <v>183.7599490124178</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>15.05</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>25.64283898898245</v>
+        <v>25.64283945628793</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>20.64747947396137</v>
+        <v>20.64747949334777</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>1.729007181179986</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.1236964163250469</v>
+        <v>-0.1236964167175224</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>39.25566949276527</v>
+        <v>39.2556696280979</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>17.85990102904315</v>
+        <v>17.85990093081092</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.9526613838198412</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.2239924766025558</v>
+        <v>0.2239924760418641</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>35.45025766256286</v>
+        <v>35.45025711397589</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>29.96303996000574</v>
+        <v>29.96304162317092</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.3175174391228578</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.03792028767282385</v>
+        <v>0.03792028803726044</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>44.43983864191284</v>
+        <v>44.43983894370405</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>17.90093397741712</v>
+        <v>17.90093422467318</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.9943424826983293</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.6450103203932613</v>
+        <v>-0.6450103227761597</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,7 +6541,7 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>39.87702634945363</v>
+        <v>39.87702630692639</v>
       </c>
       <c r="I115" s="2" t="n">
         <v>26.9258781903117</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.06877389278876844</v>
+        <v>-0.06877389264860212</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,7 +6594,7 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>28.11688305536011</v>
+        <v>28.11688252300939</v>
       </c>
       <c r="I116" s="2" t="n">
         <v>11.30793333597864</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.2227020186607662</v>
+        <v>-0.2227020182402613</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>20.5936061652221</v>
+        <v>20.59360602735167</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>14.49182781319054</v>
+        <v>14.49182761666174</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>4.021508906430247</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>39.36881415833792</v>
+        <v>39.36881429244666</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>17.25639960495843</v>
+        <v>17.25639966482964</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.6644970316679577</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-2.183333647889537</v>
+        <v>-2.183333649010883</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>51.47476529479479</v>
+        <v>51.47476533893278</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>4.786972709018599</v>
+        <v>4.786972799248487</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>1.084288657354927</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.1600339341388994</v>
+        <v>0.1600339339146319</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>129.1091885705276</v>
+        <v>129.1091885705272</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>15.65</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>37.02074664601204</v>
+        <v>37.0207174572559</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.23202572308351</v>
+        <v>15.23203335033949</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.8373586176754699</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.02321817770858725</v>
+        <v>-0.02321816858888032</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6845,7 +6845,7 @@
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>122.5825622446082</v>
+        <v>122.5825622446081</v>
       </c>
       <c r="E121" s="2" t="n">
         <v>25.3</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>26.14012148714799</v>
+        <v>26.14012168798371</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>24.16427861038929</v>
+        <v>24.16427879039361</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.2915990655167355</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.04248755113559421</v>
+        <v>-0.04248755126174975</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>120.350956251485</v>
+        <v>120.3509562514848</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>249</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>31.52889863935657</v>
+        <v>31.52889874788288</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>14.09416564606516</v>
+        <v>14.0941656048159</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>1.25176317180764</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.6847255947837869</v>
+        <v>-0.6847255953444602</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>39.1966593272096</v>
+        <v>39.19665924276629</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.17440692386337</v>
+        <v>13.1744069374196</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>1.092703328027108</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.2233572824532173</v>
+        <v>-0.2233572823270643</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>108.1222171030564</v>
+        <v>108.1222171030565</v>
       </c>
       <c r="E124" s="2" t="n">
         <v>265.5</v>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>37.2854904236905</v>
+        <v>37.28549040671761</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>17.36300254019361</v>
+        <v>17.36300254770311</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.4677438334097521</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-3.929460933697228</v>
+        <v>-3.929460933557094</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7057,7 +7057,7 @@
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>108.0471407190917</v>
+        <v>108.0471407190916</v>
       </c>
       <c r="E125" s="2" t="n">
         <v>547</v>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>34.54311418470519</v>
+        <v>34.54311415141211</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>18.7409619506133</v>
+        <v>18.74096198867686</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.2637643471107782</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-8.921718145648235</v>
+        <v>-8.921718144526871</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>100.1426058692707</v>
+        <v>100.1426058692748</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>16.75</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>43.50025562478501</v>
+        <v>43.5002556639789</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>19.65312675709144</v>
+        <v>19.65312682969188</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.1888328657471896</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.01633143832362741</v>
+        <v>-0.01633143830961276</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>20.1359595935498</v>
+        <v>20.13596032715861</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>16.93497553835291</v>
+        <v>16.93497545649658</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.6002778183225612</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.03347239843567795</v>
+        <v>-0.03347239894028564</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>45.73796497625422</v>
+        <v>45.73796494533001</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>17.22361057253819</v>
+        <v>17.22361061867297</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.4034722290199748</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>-0.2111764719525156</v>
+        <v>-0.211176471840382</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>

</xml_diff>